<commit_message>
Overhauling and improving the demo website
</commit_message>
<xml_diff>
--- a/implementation_layer/toolkit_demo_app/public/data/po-bom-example/price list.xlsx
+++ b/implementation_layer/toolkit_demo_app/public/data/po-bom-example/price list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h02317\Downloads\PO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h02317\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADEDACD7-FFAA-4207-8BB2-2600D91D3E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B0B735B-A205-420D-B083-09517D00B76C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,9 +67,6 @@
     <t>ALUMINUM PRODUCTS</t>
   </si>
   <si>
-    <t>AL-001</t>
-  </si>
-  <si>
     <t>Aluminum Angle - L Profile</t>
   </si>
   <si>
@@ -79,39 +76,24 @@
     <t>6m length</t>
   </si>
   <si>
-    <t>AL-002</t>
-  </si>
-  <si>
     <t>Aluminum Flat Bar</t>
   </si>
   <si>
-    <t>AL-003</t>
-  </si>
-  <si>
     <t>Aluminum Round Tube</t>
   </si>
   <si>
     <t>6063-T5</t>
   </si>
   <si>
-    <t>AL-004</t>
-  </si>
-  <si>
     <t>Aluminum Square Tube</t>
   </si>
   <si>
-    <t>AL-005</t>
-  </si>
-  <si>
     <t>Aluminum Channel - C Profile</t>
   </si>
   <si>
     <t>STAINLESS STEEL PRODUCTS</t>
   </si>
   <si>
-    <t>SS-001</t>
-  </si>
-  <si>
     <t>Stainless Steel Sheet - Grade 304</t>
   </si>
   <si>
@@ -121,78 +103,51 @@
     <t>per sheet</t>
   </si>
   <si>
-    <t>SS-002</t>
-  </si>
-  <si>
     <t>Stainless Steel Sheet - Grade 316</t>
   </si>
   <si>
     <t>316/1.4401</t>
   </si>
   <si>
-    <t>SS-003</t>
-  </si>
-  <si>
     <t>Stainless Steel Round Bar</t>
   </si>
   <si>
     <t>304</t>
   </si>
   <si>
-    <t>SS-004</t>
-  </si>
-  <si>
     <t>Stainless Steel Flat Bar</t>
   </si>
   <si>
-    <t>SS-005</t>
-  </si>
-  <si>
     <t>Stainless Steel Angle</t>
   </si>
   <si>
     <t>CARBON STEEL PRODUCTS</t>
   </si>
   <si>
-    <t>CS-001</t>
-  </si>
-  <si>
     <t>Seamless Carbon Steel Pipe</t>
   </si>
   <si>
     <t>ASTM A106 Gr B</t>
   </si>
   <si>
-    <t>CS-002</t>
-  </si>
-  <si>
     <t>Welded Carbon Steel Pipe</t>
   </si>
   <si>
     <t>ASTM A53 Gr B</t>
   </si>
   <si>
-    <t>CS-003</t>
-  </si>
-  <si>
     <t>Carbon Steel Plate</t>
   </si>
   <si>
     <t>ASTM A36</t>
   </si>
   <si>
-    <t>CS-004</t>
-  </si>
-  <si>
     <t>Carbon Steel Round Bar</t>
   </si>
   <si>
     <t>AISI 1045</t>
   </si>
   <si>
-    <t>CS-005</t>
-  </si>
-  <si>
     <t>Carbon Steel Square Bar</t>
   </si>
   <si>
@@ -422,6 +377,51 @@
   </si>
   <si>
     <t>Contact: sales@precisionsteel.com | Tel: +1 (412) 555-8900</t>
+  </si>
+  <si>
+    <t>MAT-2401</t>
+  </si>
+  <si>
+    <t>MAT-2402</t>
+  </si>
+  <si>
+    <t>MAT-2403</t>
+  </si>
+  <si>
+    <t>MAT-2404</t>
+  </si>
+  <si>
+    <t>MAT-2405</t>
+  </si>
+  <si>
+    <t>MAT-3567</t>
+  </si>
+  <si>
+    <t>MAT-3568</t>
+  </si>
+  <si>
+    <t>MAT-3569</t>
+  </si>
+  <si>
+    <t>MAT-3570</t>
+  </si>
+  <si>
+    <t>MAT-3571</t>
+  </si>
+  <si>
+    <t>MAT-4829</t>
+  </si>
+  <si>
+    <t>MAT-4830</t>
+  </si>
+  <si>
+    <t>MAT-4831</t>
+  </si>
+  <si>
+    <t>MAT-4832</t>
+  </si>
+  <si>
+    <t>MAT-4833</t>
   </si>
 </sst>
 </file>
@@ -974,16 +974,16 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="E8" s="3">
         <v>28.5</v>
@@ -1006,16 +1006,16 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>19</v>
+        <v>120</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="E9" s="3">
         <v>22.75</v>
@@ -1038,16 +1038,16 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>121</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E10" s="3">
         <v>35</v>
@@ -1070,16 +1070,16 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>24</v>
+        <v>122</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E11" s="3">
         <v>38.5</v>
@@ -1102,16 +1102,16 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>26</v>
+        <v>123</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="E12" s="3">
         <v>42</v>
@@ -1134,7 +1134,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
@@ -1148,16 +1148,16 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>124</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E14" s="3">
         <v>195.75</v>
@@ -1180,16 +1180,16 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>33</v>
+        <v>125</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E15" s="3">
         <v>285</v>
@@ -1212,16 +1212,16 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>36</v>
+        <v>126</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E16" s="3">
         <v>125</v>
@@ -1244,16 +1244,16 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>39</v>
+        <v>127</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E17" s="3">
         <v>95</v>
@@ -1276,16 +1276,16 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>41</v>
+        <v>128</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E18" s="3">
         <v>78.5</v>
@@ -1308,7 +1308,7 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
@@ -1322,16 +1322,16 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>44</v>
+        <v>129</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E20" s="3">
         <v>67.2</v>
@@ -1354,16 +1354,16 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>47</v>
+        <v>130</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E21" s="3">
         <v>45</v>
@@ -1386,16 +1386,16 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>50</v>
+        <v>131</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E22" s="3">
         <v>320</v>
@@ -1418,16 +1418,16 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>53</v>
+        <v>132</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E23" s="3">
         <v>55</v>
@@ -1450,16 +1450,16 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>56</v>
+        <v>133</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E24" s="3">
         <v>48</v>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="12"/>
@@ -1496,16 +1496,16 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="E26" s="3">
         <v>450</v>
@@ -1528,16 +1528,16 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="E27" s="3">
         <v>380</v>
@@ -1560,16 +1560,16 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E28" s="3">
         <v>125</v>
@@ -1592,16 +1592,16 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E29" s="3">
         <v>65</v>
@@ -1624,16 +1624,16 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E30" s="3">
         <v>72</v>
@@ -1656,7 +1656,7 @@
     </row>
     <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7"/>
@@ -1665,73 +1665,73 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="7"/>
@@ -1740,106 +1740,106 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
@@ -1848,74 +1848,74 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B54" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B55" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="B56" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="B57" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>